<commit_message>
std update and noise detection
</commit_message>
<xml_diff>
--- a/Codigos/Windows/Desvios.xlsx
+++ b/Codigos/Windows/Desvios.xlsx
@@ -1,33 +1,121 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zakie Assad\Proyecto Final\Git\MoAna\Codigos\Windows\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9882D3-6F96-4101-AC7F-459ED3C4DAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="380" yWindow="0" windowWidth="28040" windowHeight="17440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>DATA_BRUNO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_RAMIRO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_LUANA1.csv</t>
+  </si>
+  <si>
+    <t>DATA_LUCILA1.csv</t>
+  </si>
+  <si>
+    <t>DATA_AMIR1.csv</t>
+  </si>
+  <si>
+    <t>DATA_AGUSTINA1.csv</t>
+  </si>
+  <si>
+    <t>DATA_MAXIMO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_FRANCON1.csv</t>
+  </si>
+  <si>
+    <t>DATA_MARTIN1.csv</t>
+  </si>
+  <si>
+    <t>DATA_FRANCOY1.csv</t>
+  </si>
+  <si>
+    <t>DATA_CONRADO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_TOMASA1.csv</t>
+  </si>
+  <si>
+    <t>DATA_MATEO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_MANUEL1.csv</t>
+  </si>
+  <si>
+    <t>DATA_FRANCOB1.csv</t>
+  </si>
+  <si>
+    <t>DATA_MILAGROS1.csv</t>
+  </si>
+  <si>
+    <t>DATA_LISANDRO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_FRANCOBO1.csv</t>
+  </si>
+  <si>
+    <t>DATA_JUANMANUEL1.csv</t>
+  </si>
+  <si>
+    <t>DATA_AMALIA1.csv</t>
+  </si>
+  <si>
+    <t>DATA_TERE1.csv</t>
+  </si>
+  <si>
+    <t>DATA_ZAKI1.csv</t>
+  </si>
+  <si>
+    <t>DATA_LULI1.csv</t>
+  </si>
+  <si>
+    <t>HBI</t>
+  </si>
+  <si>
+    <t>PPGA</t>
+  </si>
+  <si>
+    <t>Sujeto</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,80 +134,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -419,311 +448,272 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="n">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>33</v>
       </c>
-      <c r="B1" t="n">
+      <c r="B2">
         <v>32957</v>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>DATA_BRUNO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>40</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B3">
         <v>8071</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>DATA_RAMIRO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>27</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B4">
         <v>7858</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DATA_LUANA1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>26</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B5">
         <v>4995</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>DATA_LUCILA1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>23</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B6">
         <v>23879</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DATA_AMIR1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>25</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B7">
         <v>4768</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DATA_AGUSTINA1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>23</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B8">
         <v>3822</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DATA_MAXIMO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>30</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B9">
         <v>9031</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DATA_FRANCON1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>25</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B10">
         <v>14368</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DATA_MARTIN1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>34</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B11">
         <v>14948</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DATA_FRANCOY1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>17</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B12">
         <v>2459</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>DATA_CONRADO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>23</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B13">
         <v>29923</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>DATA_TOMASA1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>25</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B14">
         <v>25875</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>DATA_MATEO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>40</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B15">
         <v>25507</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>DATA_MANUEL1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>30</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B16">
         <v>42425</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>DATA_FRANCOB1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>26</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B17">
         <v>5971</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>DATA_MILAGROS1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>25</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B18">
         <v>64972</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>DATA_LISANDRO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>31</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B19">
         <v>8385</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DATA_FRANCOBO1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
+      <c r="C19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>36</v>
       </c>
-      <c r="B19" t="n">
+      <c r="B20">
         <v>16750</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>DATA_JUANMANUEL1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
+      <c r="C20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>24</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B21">
         <v>47804</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>DATA_AMALIA1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
+      <c r="C21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>22</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B22">
         <v>9186</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>DATA_TERE1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>15</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B23">
         <v>1109</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>DATA_ZAKI1.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>28</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B24">
         <v>12579</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>DATA_LULI1.csv</t>
-        </is>
+      <c r="C24" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>